<commit_message>
changing the project structure for pyproject.toml
</commit_message>
<xml_diff>
--- a/margin_estimator_tool/output/margin_details.xlsx
+++ b/margin_estimator_tool/output/margin_details.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -600,10 +600,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20241008</v>
+        <v>20241107</v>
       </c>
       <c r="B2" t="n">
-        <v>1164.505330283922</v>
+        <v>1021.949461237886</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -616,28 +616,28 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.07931607418488845</v>
+        <v>0.01887059479827517</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1164.426014209737</v>
+        <v>1021.930590643088</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>99.94461420973757</v>
+        <v>91.56069064308842</v>
       </c>
       <c r="J2" t="n">
-        <v>1064.4814</v>
+        <v>930.3698999999995</v>
       </c>
       <c r="K2" t="n">
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>1164.426014209737</v>
+        <v>1021.930590643088</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -659,13 +659,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>852.2961336000004</v>
+        <v>840.8423766399999</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="n">
-        <v>852.2961336000004</v>
+        <v>840.8423766399999</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -717,10 +717,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20241008</v>
+        <v>20241108</v>
       </c>
       <c r="B3" t="n">
-        <v>1164.505330283922</v>
+        <v>1025.828073053841</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -733,28 +733,28 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.07931607418488845</v>
+        <v>0.01893208645041262</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1164.426014209737</v>
+        <v>1025.80914096739</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>99.94461420973757</v>
+        <v>92.40754096738991</v>
       </c>
       <c r="J3" t="n">
-        <v>1064.4814</v>
+        <v>933.4016000000006</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>1164.426014209737</v>
+        <v>1025.80914096739</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -776,13 +776,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>852.2961336000004</v>
+        <v>848.9273547199998</v>
       </c>
       <c r="S3" t="n">
         <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>852.2961336000004</v>
+        <v>848.9273547199998</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -829,123 +829,6 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>20241008</v>
-      </c>
-      <c r="B4" t="n">
-        <v>1164.505330283922</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PEQ01</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>PEQ01_HP3</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0.07931607418488845</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1164.426014209737</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>99.94461420973757</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1064.4814</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1164.426014209737</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>FILTERED_HISTORICAL_VAR_3</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Historical</t>
-        </is>
-      </c>
-      <c r="O4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>852.2961336000004</v>
-      </c>
-      <c r="S4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T4" t="n">
-        <v>852.2961336000004</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>SIMPLE_STRESS_VAR_3</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>Stress</t>
-        </is>
-      </c>
-      <c r="W4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>-0</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>EVENT_RISK_PEQ01</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="AE4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -960,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1047,11 +930,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20241008</v>
+        <v>20241107</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1164.505330283922</v>
+        <v>1021.949461237886</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1107,11 +990,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20241008</v>
+        <v>20241108</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
-        <v>1164.505330283922</v>
+        <v>1025.828073053841</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1160,66 +1043,6 @@
         </is>
       </c>
       <c r="P3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>20241008</v>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="n">
-        <v>1164.505330283922</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>20321217</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>58483525</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>PEQ01</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>PEQ01_HP3</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>203212</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>FEXD</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>